<commit_message>
20230731 16, 17, 18 한영
</commit_message>
<xml_diff>
--- a/score_card/이은선.xlsx
+++ b/score_card/이은선.xlsx
@@ -8,18 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\canaanaca\score_card\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADC4189E-8944-45CE-8F89-D80990719C09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8F7007F-676B-4ABB-8897-3955335AC307}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32295" yWindow="3300" windowWidth="17280" windowHeight="11940" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="DB" sheetId="2" r:id="rId1"/>
     <sheet name="score_card" sheetId="5" r:id="rId2"/>
     <sheet name="mock_01" sheetId="6" r:id="rId3"/>
     <sheet name="mock_02" sheetId="7" r:id="rId4"/>
+    <sheet name="mock_03" sheetId="8" r:id="rId5"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId5"/>
     <externalReference r:id="rId6"/>
     <externalReference r:id="rId7"/>
     <externalReference r:id="rId8"/>
@@ -32,6 +32,7 @@
     <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
+    <externalReference r:id="rId18"/>
   </externalReferences>
   <calcPr calcId="191029"/>
   <extLst>
@@ -54,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="69">
   <si>
     <t>번호</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -693,7 +694,25 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -717,29 +736,32 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -3322,20 +3344,20 @@
       <c r="L14" s="4"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="22"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
-      <c r="E15" s="22"/>
-      <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="22"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="22"/>
-      <c r="L15" s="22"/>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="25"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A16" s="21" t="s">
@@ -3566,31 +3588,31 @@
         <f>DB!E20</f>
         <v>0</v>
       </c>
-      <c r="D21" s="30"/>
-      <c r="E21" s="31"/>
-      <c r="F21" s="31"/>
-      <c r="G21" s="31"/>
-      <c r="H21" s="31"/>
-      <c r="I21" s="31"/>
-      <c r="J21" s="31"/>
-      <c r="K21" s="31"/>
-      <c r="L21" s="32"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="27"/>
+      <c r="F21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="27"/>
+      <c r="I21" s="27"/>
+      <c r="J21" s="27"/>
+      <c r="K21" s="27"/>
+      <c r="L21" s="28"/>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.4">
-      <c r="A22" s="33" t="s">
+      <c r="A22" s="22" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="34"/>
-      <c r="C22" s="34"/>
-      <c r="D22" s="34"/>
-      <c r="E22" s="34"/>
-      <c r="F22" s="34"/>
-      <c r="G22" s="34"/>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="34"/>
-      <c r="K22" s="34"/>
-      <c r="L22" s="35"/>
+      <c r="B22" s="23"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="23"/>
+      <c r="G22" s="23"/>
+      <c r="H22" s="23"/>
+      <c r="I22" s="23"/>
+      <c r="J22" s="23"/>
+      <c r="K22" s="23"/>
+      <c r="L22" s="24"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.4">
       <c r="A23" s="16">
@@ -3965,13 +3987,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:5" ht="18.600000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="13" t="s">
@@ -4801,28 +4823,28 @@
       </c>
     </row>
     <row r="48" spans="1:5" ht="18" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="A48" s="23" t="s">
+      <c r="A48" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B48" s="23"/>
-      <c r="C48" s="24">
+      <c r="B48" s="29"/>
+      <c r="C48" s="30">
         <f>SUM(E3:E47)</f>
         <v>84</v>
       </c>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
+      <c r="D48" s="30"/>
+      <c r="E48" s="30"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A49" s="25" t="s">
+      <c r="A49" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B49" s="25"/>
-      <c r="C49" s="26" t="str">
+      <c r="B49" s="31"/>
+      <c r="C49" s="32" t="str">
         <f>IF(C48&gt;=90,"1등급",IF(C48&gt;=80,"2등급",IF(C48&gt;=70,"3등급",IF(C48&gt;=60,"4등급","죽어라"))))</f>
         <v>2등급</v>
       </c>
-      <c r="D49" s="26"/>
-      <c r="E49" s="26"/>
+      <c r="D49" s="32"/>
+      <c r="E49" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -4834,13 +4856,13 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C3:C47">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="8" priority="1">
       <formula>B3&lt;&gt;C3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="7" priority="2">
       <formula>B3=C3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="6" priority="3">
       <formula>"IF(B3=C3)"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4858,13 +4880,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="33" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="29"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:5" ht="18.600000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A2" s="13" t="s">
@@ -5694,28 +5716,28 @@
       </c>
     </row>
     <row r="48" spans="1:5" ht="18" thickTop="1" x14ac:dyDescent="0.4">
-      <c r="A48" s="23" t="s">
+      <c r="A48" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B48" s="23"/>
-      <c r="C48" s="24">
+      <c r="B48" s="29"/>
+      <c r="C48" s="30">
         <f>SUM(E3:E47)</f>
         <v>86</v>
       </c>
-      <c r="D48" s="24"/>
-      <c r="E48" s="24"/>
+      <c r="D48" s="30"/>
+      <c r="E48" s="30"/>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A49" s="25" t="s">
+      <c r="A49" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="B49" s="25"/>
-      <c r="C49" s="26" t="str">
+      <c r="B49" s="31"/>
+      <c r="C49" s="32" t="str">
         <f>IF(C48&gt;=90,"1등급",IF(C48&gt;=80,"2등급",IF(C48&gt;=70,"3등급",IF(C48&gt;=60,"4등급","죽어라"))))</f>
         <v>2등급</v>
       </c>
-      <c r="D49" s="26"/>
-      <c r="E49" s="26"/>
+      <c r="D49" s="32"/>
+      <c r="E49" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -5727,13 +5749,906 @@
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="C3:C47">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>B3&lt;&gt;C3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>B3=C3</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>"IF(B3=C3)"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01BC82E2-CAB7-4401-B18B-0C70E24BC0BB}">
+  <dimension ref="A1:E49"/>
+  <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="5" width="8.69921875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="33" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="35"/>
+    </row>
+    <row r="2" spans="1:5" ht="18.600000000000001" thickTop="1" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="18" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="8">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6">
+        <v>1</v>
+      </c>
+      <c r="C3" s="5">
+        <v>1</v>
+      </c>
+      <c r="D3" s="5">
+        <v>2</v>
+      </c>
+      <c r="E3" s="5">
+        <f>IF(B3=C3,D3,0)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A4" s="9">
+        <v>2</v>
+      </c>
+      <c r="B4" s="7">
+        <v>1</v>
+      </c>
+      <c r="C4" s="4">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4">
+        <f t="shared" ref="E4:E47" si="0">IF(B4=C4,D4,0)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A5" s="9">
+        <v>3</v>
+      </c>
+      <c r="B5" s="7">
+        <v>5</v>
+      </c>
+      <c r="C5" s="4">
+        <v>5</v>
+      </c>
+      <c r="D5" s="4">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A6" s="9">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7">
+        <v>4</v>
+      </c>
+      <c r="C6" s="4">
+        <v>4</v>
+      </c>
+      <c r="D6" s="4">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A7" s="9">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="4">
+        <v>1</v>
+      </c>
+      <c r="D7" s="4">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A8" s="9">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7">
+        <v>4</v>
+      </c>
+      <c r="C8" s="4">
+        <v>4</v>
+      </c>
+      <c r="D8" s="4">
+        <v>3</v>
+      </c>
+      <c r="E8" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A9" s="9">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7">
+        <v>5</v>
+      </c>
+      <c r="C9" s="4">
+        <v>5</v>
+      </c>
+      <c r="D9" s="4">
+        <v>2</v>
+      </c>
+      <c r="E9" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A10" s="9">
+        <v>8</v>
+      </c>
+      <c r="B10" s="7">
+        <v>4</v>
+      </c>
+      <c r="C10" s="4">
+        <v>4</v>
+      </c>
+      <c r="D10" s="4">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A11" s="9">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7">
+        <v>3</v>
+      </c>
+      <c r="C11" s="4">
+        <v>3</v>
+      </c>
+      <c r="D11" s="4">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A12" s="9">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7">
+        <v>2</v>
+      </c>
+      <c r="C12" s="4">
+        <v>2</v>
+      </c>
+      <c r="D12" s="4">
+        <v>2</v>
+      </c>
+      <c r="E12" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A13" s="9">
+        <v>11</v>
+      </c>
+      <c r="B13" s="7">
+        <v>2</v>
+      </c>
+      <c r="C13" s="4">
+        <v>2</v>
+      </c>
+      <c r="D13" s="4">
+        <v>2</v>
+      </c>
+      <c r="E13" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A14" s="9">
+        <v>12</v>
+      </c>
+      <c r="B14" s="7">
+        <v>2</v>
+      </c>
+      <c r="C14" s="4">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4">
+        <v>2</v>
+      </c>
+      <c r="E14" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A15" s="9">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7">
+        <v>4</v>
+      </c>
+      <c r="C15" s="4">
+        <v>4</v>
+      </c>
+      <c r="D15" s="4">
+        <v>3</v>
+      </c>
+      <c r="E15" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A16" s="9">
+        <v>14</v>
+      </c>
+      <c r="B16" s="7">
+        <v>1</v>
+      </c>
+      <c r="C16" s="4">
+        <v>1</v>
+      </c>
+      <c r="D16" s="4">
+        <v>3</v>
+      </c>
+      <c r="E16" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A17" s="9">
+        <v>15</v>
+      </c>
+      <c r="B17" s="7">
+        <v>3</v>
+      </c>
+      <c r="C17" s="4">
+        <v>3</v>
+      </c>
+      <c r="D17" s="4">
+        <v>2</v>
+      </c>
+      <c r="E17" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A18" s="9">
+        <v>16</v>
+      </c>
+      <c r="B18" s="7">
+        <v>2</v>
+      </c>
+      <c r="C18" s="4">
+        <v>2</v>
+      </c>
+      <c r="D18" s="4">
+        <v>2</v>
+      </c>
+      <c r="E18" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A19" s="9">
+        <v>17</v>
+      </c>
+      <c r="B19" s="7">
+        <v>3</v>
+      </c>
+      <c r="C19" s="4">
+        <v>3</v>
+      </c>
+      <c r="D19" s="4">
+        <v>2</v>
+      </c>
+      <c r="E19" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A20" s="9">
+        <v>18</v>
+      </c>
+      <c r="B20" s="7">
+        <v>3</v>
+      </c>
+      <c r="C20" s="4">
+        <v>3</v>
+      </c>
+      <c r="D20" s="4">
+        <v>2</v>
+      </c>
+      <c r="E20" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A21" s="9">
+        <v>19</v>
+      </c>
+      <c r="B21" s="7">
+        <v>1</v>
+      </c>
+      <c r="C21" s="4">
+        <v>1</v>
+      </c>
+      <c r="D21" s="4">
+        <v>2</v>
+      </c>
+      <c r="E21" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A22" s="9">
+        <v>20</v>
+      </c>
+      <c r="B22" s="7">
+        <v>1</v>
+      </c>
+      <c r="C22" s="4">
+        <v>1</v>
+      </c>
+      <c r="D22" s="4">
+        <v>2</v>
+      </c>
+      <c r="E22" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A23" s="9">
+        <v>21</v>
+      </c>
+      <c r="B23" s="7">
+        <v>5</v>
+      </c>
+      <c r="C23" s="4">
+        <v>5</v>
+      </c>
+      <c r="D23" s="4">
+        <v>2</v>
+      </c>
+      <c r="E23" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A24" s="9">
+        <v>22</v>
+      </c>
+      <c r="B24" s="7">
+        <v>5</v>
+      </c>
+      <c r="C24" s="4">
+        <v>5</v>
+      </c>
+      <c r="D24" s="4">
+        <v>2</v>
+      </c>
+      <c r="E24" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A25" s="9">
+        <v>23</v>
+      </c>
+      <c r="B25" s="7">
+        <v>1</v>
+      </c>
+      <c r="C25" s="4">
+        <v>1</v>
+      </c>
+      <c r="D25" s="4">
+        <v>2</v>
+      </c>
+      <c r="E25" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A26" s="9">
+        <v>24</v>
+      </c>
+      <c r="B26" s="7">
+        <v>5</v>
+      </c>
+      <c r="C26" s="4">
+        <v>5</v>
+      </c>
+      <c r="D26" s="4">
+        <v>2</v>
+      </c>
+      <c r="E26" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A27" s="9">
+        <v>25</v>
+      </c>
+      <c r="B27" s="7">
+        <v>4</v>
+      </c>
+      <c r="C27" s="4">
+        <v>4</v>
+      </c>
+      <c r="D27" s="4">
+        <v>2</v>
+      </c>
+      <c r="E27" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A28" s="9">
+        <v>26</v>
+      </c>
+      <c r="B28" s="7">
+        <v>4</v>
+      </c>
+      <c r="C28" s="4">
+        <v>4</v>
+      </c>
+      <c r="D28" s="4">
+        <v>2</v>
+      </c>
+      <c r="E28" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A29" s="9">
+        <v>27</v>
+      </c>
+      <c r="B29" s="7">
+        <v>5</v>
+      </c>
+      <c r="C29" s="4">
+        <v>5</v>
+      </c>
+      <c r="D29" s="4">
+        <v>2</v>
+      </c>
+      <c r="E29" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A30" s="9">
+        <v>28</v>
+      </c>
+      <c r="B30" s="7">
+        <v>4</v>
+      </c>
+      <c r="C30" s="4">
+        <v>4</v>
+      </c>
+      <c r="D30" s="4">
+        <v>2</v>
+      </c>
+      <c r="E30" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A31" s="9">
+        <v>29</v>
+      </c>
+      <c r="B31" s="7">
+        <v>2</v>
+      </c>
+      <c r="C31" s="4">
+        <v>2</v>
+      </c>
+      <c r="D31" s="4">
+        <v>3</v>
+      </c>
+      <c r="E31" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A32" s="9">
+        <v>30</v>
+      </c>
+      <c r="B32" s="7">
+        <v>5</v>
+      </c>
+      <c r="C32" s="4">
+        <v>5</v>
+      </c>
+      <c r="D32" s="4">
+        <v>3</v>
+      </c>
+      <c r="E32" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A33" s="9">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7">
+        <v>4</v>
+      </c>
+      <c r="C33" s="4">
+        <v>4</v>
+      </c>
+      <c r="D33" s="4">
+        <v>2</v>
+      </c>
+      <c r="E33" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A34" s="9">
+        <v>32</v>
+      </c>
+      <c r="B34" s="7">
+        <v>2</v>
+      </c>
+      <c r="C34" s="4">
+        <v>2</v>
+      </c>
+      <c r="D34" s="4">
+        <v>2</v>
+      </c>
+      <c r="E34" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A35" s="9">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7">
+        <v>4</v>
+      </c>
+      <c r="C35" s="4">
+        <v>4</v>
+      </c>
+      <c r="D35" s="4">
+        <v>3</v>
+      </c>
+      <c r="E35" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A36" s="9">
+        <v>34</v>
+      </c>
+      <c r="B36" s="7">
+        <v>2</v>
+      </c>
+      <c r="C36" s="4">
+        <v>1</v>
+      </c>
+      <c r="D36" s="4">
+        <v>3</v>
+      </c>
+      <c r="E36" s="4">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A37" s="9">
+        <v>35</v>
+      </c>
+      <c r="B37" s="7">
+        <v>3</v>
+      </c>
+      <c r="C37" s="4">
+        <v>3</v>
+      </c>
+      <c r="D37" s="4">
+        <v>2</v>
+      </c>
+      <c r="E37" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A38" s="9">
+        <v>36</v>
+      </c>
+      <c r="B38" s="7">
+        <v>2</v>
+      </c>
+      <c r="C38" s="4">
+        <v>2</v>
+      </c>
+      <c r="D38" s="4">
+        <v>2</v>
+      </c>
+      <c r="E38" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A39" s="9">
+        <v>37</v>
+      </c>
+      <c r="B39" s="7">
+        <v>5</v>
+      </c>
+      <c r="C39" s="4">
+        <v>5</v>
+      </c>
+      <c r="D39" s="4">
+        <v>3</v>
+      </c>
+      <c r="E39" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A40" s="9">
+        <v>38</v>
+      </c>
+      <c r="B40" s="7">
+        <v>3</v>
+      </c>
+      <c r="C40" s="4">
+        <v>3</v>
+      </c>
+      <c r="D40" s="4">
+        <v>2</v>
+      </c>
+      <c r="E40" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A41" s="9">
+        <v>39</v>
+      </c>
+      <c r="B41" s="7">
+        <v>3</v>
+      </c>
+      <c r="C41" s="4">
+        <v>3</v>
+      </c>
+      <c r="D41" s="4">
+        <v>3</v>
+      </c>
+      <c r="E41" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A42" s="9">
+        <v>40</v>
+      </c>
+      <c r="B42" s="7">
+        <v>5</v>
+      </c>
+      <c r="C42" s="4">
+        <v>5</v>
+      </c>
+      <c r="D42" s="4">
+        <v>2</v>
+      </c>
+      <c r="E42" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A43" s="9">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7">
+        <v>5</v>
+      </c>
+      <c r="C43" s="4">
+        <v>5</v>
+      </c>
+      <c r="D43" s="4">
+        <v>2</v>
+      </c>
+      <c r="E43" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A44" s="9">
+        <v>42</v>
+      </c>
+      <c r="B44" s="7">
+        <v>4</v>
+      </c>
+      <c r="C44" s="4">
+        <v>4</v>
+      </c>
+      <c r="D44" s="4">
+        <v>2</v>
+      </c>
+      <c r="E44" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A45" s="9">
+        <v>43</v>
+      </c>
+      <c r="B45" s="7">
+        <v>3</v>
+      </c>
+      <c r="C45" s="4">
+        <v>3</v>
+      </c>
+      <c r="D45" s="4">
+        <v>3</v>
+      </c>
+      <c r="E45" s="4">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A46" s="9">
+        <v>44</v>
+      </c>
+      <c r="B46" s="7">
+        <v>4</v>
+      </c>
+      <c r="C46" s="4">
+        <v>4</v>
+      </c>
+      <c r="D46" s="4">
+        <v>2</v>
+      </c>
+      <c r="E46" s="4">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" ht="18" thickBot="1" x14ac:dyDescent="0.45">
+      <c r="A47" s="10">
+        <v>45</v>
+      </c>
+      <c r="B47" s="11">
+        <v>5</v>
+      </c>
+      <c r="C47" s="12">
+        <v>5</v>
+      </c>
+      <c r="D47" s="4">
+        <v>2</v>
+      </c>
+      <c r="E47" s="12">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" ht="18" thickTop="1" x14ac:dyDescent="0.4">
+      <c r="A48" s="29" t="s">
+        <v>42</v>
+      </c>
+      <c r="B48" s="29"/>
+      <c r="C48" s="30">
+        <f>SUM(E3:E47)</f>
+        <v>97</v>
+      </c>
+      <c r="D48" s="30"/>
+      <c r="E48" s="30"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A49" s="31" t="s">
+        <v>7</v>
+      </c>
+      <c r="B49" s="31"/>
+      <c r="C49" s="32" t="str">
+        <f>IF(C48&gt;=90,"1등급",IF(C48&gt;=80,"2등급",IF(C48&gt;=70,"3등급",IF(C48&gt;=60,"4등급","죽어라"))))</f>
+        <v>1등급</v>
+      </c>
+      <c r="D49" s="32"/>
+      <c r="E49" s="32"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A48:B48"/>
+    <mergeCell ref="C48:E48"/>
+    <mergeCell ref="A49:B49"/>
+    <mergeCell ref="C49:E49"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <conditionalFormatting sqref="C3:C47">
     <cfRule type="expression" dxfId="2" priority="1">
       <formula>B3&lt;&gt;C3</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="2">
       <formula>B3=C3</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="0" priority="3">
       <formula>"IF(B3=C3)"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>